<commit_message>
Update FAT resolution docs: root cause, permanent fix, and screenshots
</commit_message>
<xml_diff>
--- a/02. FAT_Resolution Document/S4_FAT_AXCELEFT-3245_field type conflict..xlsx
+++ b/02. FAT_Resolution Document/S4_FAT_AXCELEFT-3245_field type conflict..xlsx
@@ -273,7 +273,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -514,6 +514,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -590,6 +596,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4572000" cy="2286000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1057,9 +1093,9 @@
     </row>
     <row r="16" ht="54.95" customHeight="1">
       <c r="A16" s="16" t="n"/>
-      <c r="B16" s="81" t="inlineStr">
-        <is>
-          <t>Not available from Jira ticket export — requires RCA input from assignee (Vikas San).</t>
+      <c r="B16" s="87" t="inlineStr">
+        <is>
+          <t>Report /B2WISE/05_OS_RETRIEVE, line 323 — wrong parameter sent to the function module during conversion, causing a field type conflict.</t>
         </is>
       </c>
       <c r="C16" s="72" t="n"/>
@@ -1297,9 +1333,10 @@
     </row>
     <row r="32" ht="50.1" customHeight="1">
       <c r="A32" s="33" t="n"/>
-      <c r="B32" s="31" t="inlineStr">
-        <is>
-          <t>Not available from Jira ticket export — pending detailed resolution notes.</t>
+      <c r="B32" s="88" t="inlineStr">
+        <is>
+          <t>Corrected the parameter passed to the function module at line 323 of /B2WISE/05_OS_RETRIEVE so it matches the expected field type.
+Re-tested the conversion in /CCEJ/RURCO_FI_UPLD; the field type conflict no longer occurs.</t>
         </is>
       </c>
       <c r="C32" s="76" t="n"/>
@@ -1443,5 +1480,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" display="https://ccbji-my.sharepoint.com/:f:/r/personal/dbbk_axcel01_ccbji_co_jp/Documents/Clean Core/03. S4 Transition/02. Lift/07. Test/02. FAT_INT/02. FAT_Resolution Document?csf=1&amp;web=1&amp;e=fpvHDh" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>